<commit_message>
Time entry update: finances.xlsx [2026-04-09 16:58 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="transactions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="transactions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="settings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -475,19 +475,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>key</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
+          <t>annual_staff_cost</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>757365.08</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>annual_income_goal</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Time entry update: finances.xlsx [2026-04-09 17:12 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,6 +498,106 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>goal_901a</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>59832.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>goal_901b</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>35116.58</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>goal_902</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>goal_903</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>goal_904</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>47500</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>goal_905</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>47500</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>goal_906</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>goal_907</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>325000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>goal_910</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>175000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>goal_917</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>160000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Time entry update: finances.xlsx [2026-04-09 17:17 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -17,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -47,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,6 +466,43 @@
           <t>notes</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>46118</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>25225.76</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>904</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Cities for People</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FG | Talls 1st payment of $62,440; RTL credit is 50% of $101,000 less $60 bank fee</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Time entry update: finances.xlsx [2026-04-09 17:18 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -502,7 +502,11 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -535,7 +539,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>872500</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Time entry update: finances.xlsx [2026-04-09 17:19 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,6 +507,43 @@
           <t>None</t>
         </is>
       </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>46111</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>903</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Short-term Projects</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Clark Contracting Services - DS Speaking Fee</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Time entry update: finances.xlsx [2026-04-09 17:21 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,7 +543,48 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46120</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>43761.69</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>910</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ClimateWorks Code Research</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>First payment invoiced, recv'd by HQ via check on 8 April</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Time entry update: finances.xlsx [2026-04-09 17:22 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,7 +584,48 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>46121</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>131205</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>910</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ClimateWorks Code Research</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Second payment, not yet invoiced</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Contracted</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Time entry update: finances.xlsx [2026-04-09 17:27 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -625,7 +625,48 @@
           <t>Contracted</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>46121</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>904</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Cities for People</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>KPF C4P partnership, RTL share</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Verbal</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Time entry update: finances.xlsx [2026-04-09 17:28 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -666,7 +666,48 @@
           <t>Verbal</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>46121</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>40000</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>917</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Commissioned Research</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Verbal commitments from RWDI &amp; CPP to Wind Guide, per RD</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Verbal</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Time entry update: finances.xlsx [2026-04-09 17:29 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -707,7 +707,48 @@
           <t>Verbal</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>46121</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>917</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Commissioned Research</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Outdoor Comfort Guide, per RD</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Time entry update: finances.xlsx [2026-04-09 17:30 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -830,7 +830,48 @@
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>46112</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>48363</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>901b</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Canada Research Office</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>City of Toronto building scorecard bid, submitted 31 March</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update: finances.xlsx [2026-04-09 19:01 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -871,7 +871,48 @@
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>46096</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>47500</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>905</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Sustainability Program</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>constructsteel partnership, full payment, RTL share</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update: finances.xlsx [2026-04-09 19:03 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -912,7 +912,48 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>25225.76</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>904</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Cities for People</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>FG | Talls 2nd payment, due August 2026, RTL share</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Invoiced</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update: finances.xlsx [2026-04-09 20:30 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -953,7 +953,11 @@
           <t>Invoiced</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1086,7 +1090,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>160000</v>
+        <v>165000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: finances.xlsx [2026-04-13 15:34 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -958,6 +958,39 @@
           <t>nan</t>
         </is>
       </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>855</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>910</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>ClimateWorks Code Research</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Chinese standard code purchase</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update: finances.xlsx [2026-04-13 15:46 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -989,8 +989,49 @@
           <t>Chinese standard code purchase</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>46098</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>936.14</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>903</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Short-term Projects</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>DS trip reimbursement, covered by Clark $1k payment</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update: finances.xlsx [2026-04-23 16:29 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -1030,8 +1030,16 @@
           <t>DS trip reimbursement, covered by Clark $1k payment</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1044,7 +1052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1070,100 +1078,80 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>goal_901a</t>
+          <t>goal_901b</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>59832.1</v>
+        <v>35116.58</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>goal_901b</t>
+          <t>goal_903</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>35116.58</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>goal_902</t>
+          <t>goal_904</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20000</v>
+        <v>47500</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>goal_903</t>
+          <t>goal_905</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50000</v>
+        <v>47500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>goal_904</t>
+          <t>goal_906</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>47500</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>goal_905</t>
+          <t>goal_907</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>47500</v>
+        <v>325000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>goal_906</t>
+          <t>goal_910</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>30000</v>
+        <v>175000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>goal_907</t>
+          <t>goal_917</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>325000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>goal_910</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>175000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>goal_917</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
         <v>165000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update: finances.xlsx [2026-05-15 19:23 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -743,11 +743,7 @@
           <t>Outdoor Comfort Guide, per RD</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>nan</t>
@@ -825,11 +821,7 @@
           <t>Bird Strike Prevention Guide, per RD</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>nan</t>
@@ -841,36 +833,32 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>46112</v>
+        <v>46154</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>48363</v>
+        <v>2106.7</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>901b</t>
+          <t>904</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Canada Research Office</t>
+          <t>Cities for People</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>City of Toronto building scorecard bid, submitted 31 March</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
+          <t>DS trip to Brazil</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>nan</t>

</xml_diff>

<commit_message>
Update: finances.xlsx [2026-05-15 19:24 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>47500</v>
+        <v>77500</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -892,7 +892,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>constructsteel partnership, full payment, RTL share</t>
+          <t>constructsteel partnership, full payment, RTL share; upped to $77.5k per Martus, 15 May 2026</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">

</xml_diff>

<commit_message>
Update: finances.xlsx [2026-06-30 20:47 UTC]
</commit_message>
<xml_diff>
--- a/finances.xlsx
+++ b/finances.xlsx
@@ -677,7 +677,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46121</v>
+        <v>46197</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>40000</v>
+        <v>20000</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -699,12 +699,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Verbal commitments from RWDI &amp; CPP to Wind Guide, per RD</t>
+          <t>RWDI for Wind Engineering Guide</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Verbal</t>
+          <t>Invoiced</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">

</xml_diff>